<commit_message>
fix: corrige tempo de empresa, adiciona testes estatisticos e motivos de desligamento
- ETL: remove caminho absoluto do Windows e celulas duplicadas
- ETL: recalcula tempo_empresa_anos a partir das datas (desligados eram contados ate hoje)
- ETL: normaliza data_desligamento e adiciona validacao de coerencia do tempo de empresa
- EDA: teste qui-quadrado e V de Cramer em cada recorte, com tabela-resumo
- EDA: nova secao de motivos de desligamento (voluntario x involuntario)
- EDA: conclusao de promocao, nota sobre circularidade do indice de fatores
- EDA: conclusoes, decisoes e KPIs revisados; notebooks executados do inicio ao fim
- README e requirements atualizados (versoes reais + scipy)
</commit_message>
<xml_diff>
--- a/powerBi/People_Analytics_Resumo_Executivo.xlsx
+++ b/powerBi/People_Analytics_Resumo_Executivo.xlsx
@@ -16,6 +16,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promoção" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equilíbrio" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fatores Acumulados" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motivos de Desligamento" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testes Estatísticos" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -535,7 +537,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6.033333333333333</v>
+        <v>5.8625</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -555,6 +557,366 @@
       <c r="C8" t="inlineStr">
         <is>
           <t>reais</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>motivo_desligamento</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>total_desligados</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>participacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Nova oportunidade profissional</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>53</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.1640866873065016</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Qualidade de vida</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.1547987616099071</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Falta de perspectiva de crescimento</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>46</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.1424148606811146</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Mudança de cidade</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>46</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.1424148606811146</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Desempenho abaixo do esperado</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>45</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.1393188854489164</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Remuneração e benefícios</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>42</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.130030959752322</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Reestruturação organizacional</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>41</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.1269349845201238</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>variavel</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>qui_quadrado</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>graus_liberdade</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>p_valor</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>v_cramer</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>significativo_5pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Tempo de empresa</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>76.27</v>
+      </c>
+      <c r="C2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Acúmulo de fatores</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>51.88</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Satisfação no trabalho</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>16.69</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Equilíbrio vida-trabalho</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0312</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Promoção nos últimos 5 anos</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0354</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Horas extras</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.2019</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Área</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7.63</v>
+      </c>
+      <c r="C8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Faixa salarial</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.3771</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -923,13 +1285,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="C2" t="n">
-        <v>73</v>
+        <v>115</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3187772925764192</v>
+        <v>0.4693877551020408</v>
       </c>
     </row>
     <row r="3">
@@ -939,13 +1301,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="C3" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3101604278074866</v>
+        <v>0.295</v>
       </c>
     </row>
     <row r="4">
@@ -955,13 +1317,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C4" t="n">
         <v>55</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2208835341365462</v>
+        <v>0.2226720647773279</v>
       </c>
     </row>
     <row r="5">
@@ -971,13 +1333,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="C5" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2508474576271186</v>
+        <v>0.2222222222222222</v>
       </c>
     </row>
     <row r="6">
@@ -987,13 +1349,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C6" t="n">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2625</v>
+        <v>0.1363636363636364</v>
       </c>
     </row>
   </sheetData>
@@ -1364,13 +1726,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C2" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1466666666666667</v>
+        <v>0.1081081081081081</v>
       </c>
     </row>
     <row r="3">
@@ -1380,13 +1742,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="C3" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="D3" t="n">
-        <v>0.232620320855615</v>
+        <v>0.2081081081081081</v>
       </c>
     </row>
     <row r="4">
@@ -1396,13 +1758,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>398</v>
+        <v>384</v>
       </c>
       <c r="C4" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2839195979899498</v>
+        <v>0.2916666666666667</v>
       </c>
     </row>
     <row r="5">
@@ -1412,13 +1774,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>278</v>
+        <v>298</v>
       </c>
       <c r="C5" t="n">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3633093525179856</v>
+        <v>0.3959731543624161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: evolucao do turnover, modelo logistico e melhorias de portfolio
- README reescrito com resumo executivo, resultados e recomendacoes priorizadas
- EDA: turnover anual e mensal (headcount medio), voluntario x involuntario
- Novo notebook 03: regressao logistica da saida voluntaria (odds ratio, IC 95%, AUC)
- src/people_analytics.py: funcoes reutilizaveis (taxas, teste qui-quadrado, graficos)
- Graficos com titulos que comunicam a conclusao e p-valor no subtitulo
- data/ separado em raw e processed; novas bases para o Power BI
- powerBi/GUIA_DASHBOARD.md com modelo de dados, medidas DAX e layout
- ETL: remove titulos soltos e imports sem uso
- requirements com statsmodels e scikit-learn
</commit_message>
<xml_diff>
--- a/powerBi/People_Analytics_Resumo_Executivo.xlsx
+++ b/powerBi/People_Analytics_Resumo_Executivo.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fatores Acumulados" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motivos de Desligamento" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testes Estatísticos" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolução Anual" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -925,6 +926,252 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>dias_observados</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>headcount_inicio</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>headcount_fim</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>headcount_medio</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>admissoes</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>desligamentos</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>desligamentos_voluntarios</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>desligamentos_involuntarios</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>turnover_anualizado</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>turnover_voluntario_anualizado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B2" t="n">
+        <v>365</v>
+      </c>
+      <c r="C2" t="n">
+        <v>745</v>
+      </c>
+      <c r="D2" t="n">
+        <v>787</v>
+      </c>
+      <c r="E2" t="n">
+        <v>766</v>
+      </c>
+      <c r="F2" t="n">
+        <v>83</v>
+      </c>
+      <c r="G2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I2" t="n">
+        <v>14</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.05221932114882506</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.0339425587467363</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B3" t="n">
+        <v>365</v>
+      </c>
+      <c r="C3" t="n">
+        <v>787</v>
+      </c>
+      <c r="D3" t="n">
+        <v>849</v>
+      </c>
+      <c r="E3" t="n">
+        <v>818</v>
+      </c>
+      <c r="F3" t="n">
+        <v>109</v>
+      </c>
+      <c r="G3" t="n">
+        <v>47</v>
+      </c>
+      <c r="H3" t="n">
+        <v>34</v>
+      </c>
+      <c r="I3" t="n">
+        <v>13</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.05745721271393643</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.04156479217603912</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B4" t="n">
+        <v>366</v>
+      </c>
+      <c r="C4" t="n">
+        <v>849</v>
+      </c>
+      <c r="D4" t="n">
+        <v>896</v>
+      </c>
+      <c r="E4" t="n">
+        <v>872.5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>107</v>
+      </c>
+      <c r="G4" t="n">
+        <v>60</v>
+      </c>
+      <c r="H4" t="n">
+        <v>46</v>
+      </c>
+      <c r="I4" t="n">
+        <v>14</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.06858001784959369</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.05257801368468849</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B5" t="n">
+        <v>365</v>
+      </c>
+      <c r="C5" t="n">
+        <v>897</v>
+      </c>
+      <c r="D5" t="n">
+        <v>943</v>
+      </c>
+      <c r="E5" t="n">
+        <v>920</v>
+      </c>
+      <c r="F5" t="n">
+        <v>135</v>
+      </c>
+      <c r="G5" t="n">
+        <v>88</v>
+      </c>
+      <c r="H5" t="n">
+        <v>64</v>
+      </c>
+      <c r="I5" t="n">
+        <v>24</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.09565217391304348</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.06956521739130435</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B6" t="n">
+        <v>252</v>
+      </c>
+      <c r="C6" t="n">
+        <v>942</v>
+      </c>
+      <c r="D6" t="n">
+        <v>877</v>
+      </c>
+      <c r="E6" t="n">
+        <v>909.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>22</v>
+      </c>
+      <c r="G6" t="n">
+        <v>88</v>
+      </c>
+      <c r="H6" t="n">
+        <v>67</v>
+      </c>
+      <c r="I6" t="n">
+        <v>21</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.1401432847282215</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.1067000008726232</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>